<commit_message>
Another go at sorting the row heights.
</commit_message>
<xml_diff>
--- a/ExcelDynamicCase/ExcelDynamicCase.xlsx
+++ b/ExcelDynamicCase/ExcelDynamicCase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29005"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29107"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harry\source\repos\ExcelDynamicCase\ExcelDynamicCase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FCC652-191B-436A-AAB5-CF51C563C7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99997F44-9079-4003-9780-18C9ACE6F193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="38700" windowHeight="15885" activeTab="1" xr2:uid="{A4107E39-ADFC-428B-BEC0-F1C599043212}"/>
+    <workbookView xWindow="12090" yWindow="1905" windowWidth="20685" windowHeight="18195" activeTab="1" xr2:uid="{A4107E39-ADFC-428B-BEC0-F1C599043212}"/>
   </bookViews>
   <sheets>
     <sheet name="Workings" sheetId="1" r:id="rId1"/>
@@ -146,7 +146,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -158,77 +158,12 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -238,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
@@ -248,31 +183,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -684,7 +598,7 @@
       </c>
     </row>
     <row r="17" spans="2:10" ht="57" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C17" s="6"/>
@@ -693,39 +607,39 @@
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
-      <c r="I17" s="7"/>
+      <c r="I17" s="6"/>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B18" s="8"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="10"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
       <c r="J18" s="2"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B19" s="8"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="10"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
       <c r="J19" s="2"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.4">
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="13"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
       <c r="J20" s="2"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.4">
@@ -848,7 +762,7 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="1">
-    <mergeCell ref="B17:I20"/>
+    <mergeCell ref="B17:I17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Another go at this.
</commit_message>
<xml_diff>
--- a/ExcelDynamicCase/ExcelDynamicCase.xlsx
+++ b/ExcelDynamicCase/ExcelDynamicCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harry\source\repos\ExcelDynamicCase\ExcelDynamicCase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99997F44-9079-4003-9780-18C9ACE6F193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F9A61E-8E49-484E-85F3-FE5F2FA474A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12090" yWindow="1905" windowWidth="20685" windowHeight="18195" activeTab="1" xr2:uid="{A4107E39-ADFC-428B-BEC0-F1C599043212}"/>
   </bookViews>
@@ -183,11 +183,11 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -761,9 +761,6 @@
     </row>
   </sheetData>
   <dataConsolidate/>
-  <mergeCells count="1">
-    <mergeCell ref="B17:I17"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>